<commit_message>
feat: tabla dinamica - ventas por vendedor y departamento
</commit_message>
<xml_diff>
--- a/EXCEL/Base-Datos-Empleados-Junio2026.xlsx
+++ b/EXCEL/Base-Datos-Empleados-Junio2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1d86eecf8daf4f0d/Documents/SQL Server Management Studio 22/Tienda-sqlserver/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{175B8AB0-EBA2-4AD5-A367-B39C1A612A2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{175B8AB0-EBA2-4AD5-A367-B39C1A612A2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{493D188E-E394-4A2F-A6C8-7B17E52647E4}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="11772" windowHeight="12240" xr2:uid="{C7DED14F-EBCD-4FC5-8DA2-1D197698C553}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="43">
   <si>
     <t>BASE DE DATOS DE EMPLEADOS - JUNIO 2026</t>
   </si>
@@ -136,13 +136,80 @@
   </si>
   <si>
     <t xml:space="preserve">Busqueda Exacta </t>
+  </si>
+  <si>
+    <r>
+      <t>¿Qué es VLOOKUP?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Busca un valor en una tabla y devuelve información relacionada.</t>
+    </r>
+  </si>
+  <si>
+    <t>Es como buscar el nombre de un estudiante y que Excel te diga automáticamente su nota.</t>
+  </si>
+  <si>
+    <t>Qué es SUMIF? Suma valores que cumplen una condición específica. Ejemplo: "Suma solo las ventas del departamento de Tecnología" me refiero mandame algo asi como esto</t>
+  </si>
+  <si>
+    <r>
+      <t>¿Qué es SUMIF?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Suma valores que cumplen una condición específica.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Ejemplo: </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"Suma solo las ventas del departamento de Tecnología"</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">A </t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUMIF-Salario por Departamento </t>
+  </si>
+  <si>
+    <t>Contabilidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recursos Humanos </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -159,6 +226,7 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
       <color rgb="FFC00000"/>
       <name val="Calibri"/>
@@ -166,15 +234,28 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FFC00000"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFF8F8F6"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -199,8 +280,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -223,33 +310,62 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -562,62 +678,73 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF30D6E9-7070-40B6-B498-6013A8D439CF}">
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:O28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="5" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="4">
+      <c r="G3" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
+      <c r="M3" s="18"/>
+      <c r="N3" s="18"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A4" s="3">
         <v>101</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -626,15 +753,16 @@
       <c r="C4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="15">
         <v>45000</v>
       </c>
       <c r="E4" s="1">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="4">
+      <c r="G4" s="9"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
         <v>102</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -643,15 +771,26 @@
       <c r="C5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="15">
         <v>32000</v>
       </c>
       <c r="E5" s="1">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="4">
+      <c r="G5" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="H5" s="19"/>
+      <c r="I5" s="19"/>
+      <c r="J5" s="19"/>
+      <c r="K5" s="19"/>
+      <c r="L5" s="19"/>
+      <c r="M5" s="19"/>
+      <c r="N5" s="19"/>
+      <c r="O5" s="19"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A6" s="3">
         <v>103</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -660,15 +799,15 @@
       <c r="C6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="15">
         <v>38000</v>
       </c>
       <c r="E6" s="1">
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="4">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A7" s="3">
         <v>104</v>
       </c>
       <c r="B7" s="1" t="s">
@@ -677,15 +816,15 @@
       <c r="C7" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="1">
+      <c r="D7" s="15">
         <v>52000</v>
       </c>
       <c r="E7" s="1">
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="4">
+    <row r="8" spans="1:15" ht="15" x14ac:dyDescent="0.35">
+      <c r="A8" s="3">
         <v>105</v>
       </c>
       <c r="B8" s="1" t="s">
@@ -694,15 +833,18 @@
       <c r="C8" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="15">
         <v>41000</v>
       </c>
       <c r="E8" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="4">
+      <c r="G8" s="10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
         <v>106</v>
       </c>
       <c r="B9" s="1" t="s">
@@ -711,15 +853,15 @@
       <c r="C9" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9" s="15">
         <v>35000</v>
       </c>
       <c r="E9" s="1">
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="4">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
         <v>107</v>
       </c>
       <c r="B10" s="1" t="s">
@@ -728,15 +870,18 @@
       <c r="C10" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="15">
         <v>29000</v>
       </c>
       <c r="E10" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="4">
+      <c r="G10" s="7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A11" s="3">
         <v>108</v>
       </c>
       <c r="B11" s="1" t="s">
@@ -745,15 +890,16 @@
       <c r="C11" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D11" s="1">
+      <c r="D11" s="15">
         <v>60000</v>
       </c>
       <c r="E11" s="1">
         <v>10</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="4">
+      <c r="G11" s="9"/>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A12" s="3">
         <v>109</v>
       </c>
       <c r="B12" s="1" t="s">
@@ -762,15 +908,18 @@
       <c r="C12" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="15">
         <v>43000</v>
       </c>
       <c r="E12" s="1">
         <v>6</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="4">
+      <c r="G12" s="9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A13" s="3">
         <v>110</v>
       </c>
       <c r="B13" s="1" t="s">
@@ -779,57 +928,58 @@
       <c r="C13" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13" s="15">
         <v>31000</v>
       </c>
       <c r="E13" s="1">
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="3" t="s">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A15" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="11" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>26</v>
       </c>
       <c r="B16" s="2">
         <v>101</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="7" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="11" t="str">
+      <c r="B17" s="8" t="str">
         <f>VLOOKUP(B16,A4:E13,2,0)</f>
         <v xml:space="preserve">Edwin Villar </v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" s="7" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E17" s="16"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B18" s="11" t="str">
+      <c r="B18" s="8" t="str">
         <f>VLOOKUP(B16,A4:E13,3,0)</f>
         <v xml:space="preserve">Tecnologia </v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="7" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>9</v>
       </c>
@@ -837,11 +987,11 @@
         <f>VLOOKUP(B16,A4:E13,4,0)</f>
         <v>45000</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="7" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>28</v>
       </c>
@@ -849,14 +999,73 @@
         <f>VLOOKUP(B16,A4:E13,5,0)</f>
         <v>3</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" s="7" t="s">
         <v>33</v>
       </c>
     </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="12" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="B23" s="2"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="15">
+        <f>SUMIF(C4:C13,"Tecnologia",D4:D13)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="B25" s="15">
+        <f>SUMIF(C4:C13,"Ventas",D4:D13)</f>
+        <v>67000</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B26" s="15">
+        <f>SUMIF(C4:C13,"Contabilidad",D4:D13)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B27" s="15">
+        <f>SUMIF(C4:C13,"Marketing",D4:D13)</f>
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" s="15">
+        <f>SUMIF(C4:C13,"Recursos Humanos",D4:D13)</f>
+        <v>38000</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="3">
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="G3:N3"/>
+    <mergeCell ref="G5:O5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>